<commit_message>
Added New test for create new event feature
</commit_message>
<xml_diff>
--- a/src/main/resources/TestData/TestData.xlsx
+++ b/src/main/resources/TestData/TestData.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PlaywrightUIFramework\src\main\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{626CE912-31D5-440B-9364-7D31D273914D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D67BF747-7B39-41E0-9B89-5DA6C8AE28C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{887D23A3-3DFA-484D-98F1-193FC5040552}"/>
   </bookViews>
   <sheets>
-    <sheet name="TestDataUI" sheetId="1" r:id="rId1"/>
+    <sheet name="TestData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,14 +34,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>TestCaseId</t>
   </si>
   <si>
-    <t>RunFlag</t>
-  </si>
-  <si>
     <t>EventName</t>
   </si>
   <si>
@@ -66,12 +63,6 @@
     <t>TotalSeats</t>
   </si>
   <si>
-    <t>TC001</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>Test Summit AI</t>
   </si>
   <si>
@@ -88,6 +79,9 @@
   </si>
   <si>
     <t>2026-10-22T18:00</t>
+  </si>
+  <si>
+    <t>TC01</t>
   </si>
 </sst>
 </file>
@@ -469,10 +463,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{575E3BFA-90CF-4872-A210-D7483E732027}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="20.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -500,39 +494,33 @@
       <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>17</v>
+      <c r="H2" s="1">
+        <v>500</v>
       </c>
       <c r="I2" s="1">
-        <v>500</v>
-      </c>
-      <c r="J2" s="1">
         <v>100</v>
       </c>
     </row>

</xml_diff>